<commit_message>
Ajustes varios Layout, lógica añadida para post migración +falta testear, ajuste mobile lambda scroll intermedio para detectar form
</commit_message>
<xml_diff>
--- a/data/Lead_information_Formulario_Argentina_Main.xlsx
+++ b/data/Lead_information_Formulario_Argentina_Main.xlsx
@@ -486,38 +486,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.chevrolet.com.ar/plan-chevrolet/sonic</t>
+          <t>https://www.chevrolet.com.ar/camionetas-suv/sonic/accesorios/formulario</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/pda-carpages?model=sonic</t>
+          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/accesorios?model=sonic</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Valeria</t>
+          <t>Isabella Gabriel</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Vega Pinto</t>
+          <t>Navarro</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>27005556</t>
+          <t>66513095</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2219595569</t>
+          <t>3819583640</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>valeriavegapinto_ar27@mrm.com</t>
+          <t>isabellagabrielnavarro_ar17@mrm.com</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -529,38 +529,38 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.chevrolet.com.ar/financiamiento-autos-corporativos/rural</t>
+          <t>https://www.chevrolet.com.ar/plan-chevrolet/spin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/productor-rural?model=servicios</t>
+          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/pda-carpages?model=spin</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Gonzalo</t>
+          <t>Diego Ana</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Cabrera Gonzalez</t>
+          <t>Romero</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>26221522</t>
+          <t>96918935</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2615501222</t>
+          <t>2998371013</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>gonzalocabreragonzalez.ar12@mrm.com</t>
+          <t>diegoanaromero_ar65@mrm.com</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -572,38 +572,38 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.chevrolet.com.ar/hibridos/captiva-phev</t>
+          <t>https://www.chevrolet.com.ar/financiamiento-autos-corporativos/alquiler</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/captiva-hibrida?model=captiva%20hibrida</t>
+          <t>https://secure-developments.com/commonwealth/argentina/gm_forms/servicios-alquiler?model=servicios</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Nicolás Claudia</t>
+          <t>Carlos Gabriela</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Salazar Ramos</t>
+          <t>Serrano</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>12384516</t>
+          <t>37954196</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2619717410</t>
+          <t>3511783694</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>nicolasclaudiasalazarramos_ar33@mrm.com</t>
+          <t>carlosgabrielaserrano_ar24@mrm.com</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -626,27 +626,27 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Héctor Emilio</t>
+          <t>Florencia</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Reyes Martinez</t>
+          <t>Rojas Flores</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>15787680</t>
+          <t>19204255</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2218191542</t>
+          <t>3518649048</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>hectoremilioreyesmartinez_ar59@mrm.com</t>
+          <t>florenciarojasflores.ar39@mrm.com</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>

</xml_diff>